<commit_message>
Add 0.4.0 recent jobs dashboard
</commit_message>
<xml_diff>
--- a/extension/templates/custom-job-template.xlsx
+++ b/extension/templates/custom-job-template.xlsx
@@ -230,7 +230,6 @@
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="64" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -244,11 +243,6 @@
           <t>Source string</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="3">
@@ -261,11 +255,6 @@
           <t>Example category heading to translate</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="3">
-        <is>
-          <t>Replace this example row.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="3">
@@ -278,11 +267,6 @@
           <t>Example refiner label</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr" s="3">
-        <is>
-          <t>Replace this example row.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr" s="3">
@@ -295,11 +279,6 @@
           <t/>
         </is>
       </c>
-      <c r="C4" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="3">
@@ -312,11 +291,6 @@
           <t/>
         </is>
       </c>
-      <c r="C5" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="3">
@@ -329,11 +303,6 @@
           <t/>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="3">
@@ -346,11 +315,6 @@
           <t/>
         </is>
       </c>
-      <c r="C7" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="3">
@@ -363,11 +327,6 @@
           <t/>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="3">
@@ -380,11 +339,6 @@
           <t/>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="3">
@@ -397,11 +351,6 @@
           <t/>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="3">
@@ -414,11 +363,6 @@
           <t/>
         </is>
       </c>
-      <c r="C11" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="3">
@@ -431,11 +375,6 @@
           <t/>
         </is>
       </c>
-      <c r="C12" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="3">
@@ -448,11 +387,6 @@
           <t/>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="3">
@@ -465,11 +399,6 @@
           <t/>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr" s="3">
@@ -482,11 +411,6 @@
           <t/>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="3">
@@ -499,11 +423,6 @@
           <t/>
         </is>
       </c>
-      <c r="C16" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="3">
@@ -516,11 +435,6 @@
           <t/>
         </is>
       </c>
-      <c r="C17" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="3">
@@ -533,11 +447,6 @@
           <t/>
         </is>
       </c>
-      <c r="C18" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr" s="3">
@@ -550,11 +459,6 @@
           <t/>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr" s="3">
@@ -567,11 +471,6 @@
           <t/>
         </is>
       </c>
-      <c r="C20" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr" s="3">
@@ -584,11 +483,6 @@
           <t/>
         </is>
       </c>
-      <c r="C21" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr" s="3">
@@ -601,11 +495,6 @@
           <t/>
         </is>
       </c>
-      <c r="C22" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr" s="3">
@@ -618,11 +507,6 @@
           <t/>
         </is>
       </c>
-      <c r="C23" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr" s="3">
@@ -635,11 +519,6 @@
           <t/>
         </is>
       </c>
-      <c r="C24" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr" s="3">
@@ -652,11 +531,6 @@
           <t/>
         </is>
       </c>
-      <c r="C25" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr" s="3">
@@ -669,11 +543,6 @@
           <t/>
         </is>
       </c>
-      <c r="C26" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr" s="3">
@@ -686,11 +555,6 @@
           <t/>
         </is>
       </c>
-      <c r="C27" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr" s="3">
@@ -703,11 +567,6 @@
           <t/>
         </is>
       </c>
-      <c r="C28" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr" s="3">
@@ -720,11 +579,6 @@
           <t/>
         </is>
       </c>
-      <c r="C29" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr" s="3">
@@ -737,11 +591,6 @@
           <t/>
         </is>
       </c>
-      <c r="C30" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr" s="3">
@@ -754,11 +603,6 @@
           <t/>
         </is>
       </c>
-      <c r="C31" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr" s="3">
@@ -771,11 +615,6 @@
           <t/>
         </is>
       </c>
-      <c r="C32" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr" s="3">
@@ -788,11 +627,6 @@
           <t/>
         </is>
       </c>
-      <c r="C33" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr" s="3">
@@ -805,11 +639,6 @@
           <t/>
         </is>
       </c>
-      <c r="C34" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr" s="3">
@@ -822,11 +651,6 @@
           <t/>
         </is>
       </c>
-      <c r="C35" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr" s="3">
@@ -839,11 +663,6 @@
           <t/>
         </is>
       </c>
-      <c r="C36" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr" s="3">
@@ -856,11 +675,6 @@
           <t/>
         </is>
       </c>
-      <c r="C37" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr" s="3">
@@ -873,11 +687,6 @@
           <t/>
         </is>
       </c>
-      <c r="C38" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr" s="3">
@@ -890,11 +699,6 @@
           <t/>
         </is>
       </c>
-      <c r="C39" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr" s="3">
@@ -907,11 +711,6 @@
           <t/>
         </is>
       </c>
-      <c r="C40" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr" s="3">
@@ -924,11 +723,6 @@
           <t/>
         </is>
       </c>
-      <c r="C41" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr" s="3">
@@ -941,11 +735,6 @@
           <t/>
         </is>
       </c>
-      <c r="C42" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr" s="3">
@@ -958,11 +747,6 @@
           <t/>
         </is>
       </c>
-      <c r="C43" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr" s="3">
@@ -975,11 +759,6 @@
           <t/>
         </is>
       </c>
-      <c r="C44" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr" s="3">
@@ -992,11 +771,6 @@
           <t/>
         </is>
       </c>
-      <c r="C45" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr" s="3">
@@ -1009,11 +783,6 @@
           <t/>
         </is>
       </c>
-      <c r="C46" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr" s="3">
@@ -1026,11 +795,6 @@
           <t/>
         </is>
       </c>
-      <c r="C47" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr" s="3">
@@ -1043,11 +807,6 @@
           <t/>
         </is>
       </c>
-      <c r="C48" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr" s="3">
@@ -1060,11 +819,6 @@
           <t/>
         </is>
       </c>
-      <c r="C49" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr" s="3">
@@ -1073,11 +827,6 @@
         </is>
       </c>
       <c r="B50" t="inlineStr" s="3">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr" s="3">
         <is>
           <t/>
         </is>

</xml_diff>